<commit_message>
Clean rebuild and production deployment prep
</commit_message>
<xml_diff>
--- a/public/templates/ceter-products-import-template.xlsx
+++ b/public/templates/ceter-products-import-template.xlsx
@@ -39,97 +39,177 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
+          <t>mpn</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>sku</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
           <t>price_kes</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>cost_price_kes</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>supplier_name</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>supplier_lead_time_days</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>reorder_level</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>reorder_quantity</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
         <is>
           <t>condition</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>stock_status</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>stock_quantity</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>images</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>specs</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>is_featured</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>is_published</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Lenovo ThinkPad T14 Gen 3</t>
+          <t>Kyocera ECOSYS M2040dn</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>lenovo-thinkpad-t14-gen-3</t>
+          <t>kyocera-ecosys-m2040dn</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Business laptop with Ryzen 5, 16GB RAM, and 512GB SSD.</t>
+          <t>Mono multifunction laser printer for office teams.</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>laptops</t>
+          <t>multifunction-printers</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>lenovo</t>
+          <t>kyocera</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>145000</t>
+          <t>1102S33NL0</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
+          <t>PRN-KYO-M2040DN</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>85000</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>62000</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Local distributor</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
           <t>refurbished</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="O2" t="inlineStr">
         <is>
           <t>in_stock</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="P2" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>https://example.com/thinkpad-front.jpg;https://example.com/thinkpad-side.jpg</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>CPU: Ryzen 5; RAM: 16GB; Storage: 512GB SSD</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>/product-placeholder.svg</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>Functions: Print Copy Scan; Speed: 40ppm; Paper size: A4</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
         <is>
           <t>true</t>
         </is>
@@ -138,22 +218,22 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>HP EliteDisplay E243</t>
+          <t>HP LaserJet Pro M404dn</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>hp-elitedisplay-e243</t>
+          <t>hp-laserjet-pro-m404dn</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>23.8 inch FHD office monitor with adjustable stand.</t>
+          <t>A4 mono laser printer with duplex and network printing.</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>monitors</t>
+          <t>laser-printers</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -163,37 +243,77 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>24000</t>
+          <t>W1A53A</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
+          <t>PRN-HP-M404DN</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>42000</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
           <t>new</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="O3" t="inlineStr">
         <is>
           <t>backorder</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="P3" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>https://example.com/e243.jpg</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Size: 23.8 inch; Resolution: 1080p</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>/product-placeholder.svg</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>Functions: Print; Speed: 38ppm; Paper size: A4</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
         <is>
           <t>false</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>true</t>
         </is>
       </c>
     </row>
@@ -309,24 +429,24 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>price_kes</t>
+          <t>mpn</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Required</t>
+          <t>Optional</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Whole number in KES, greater than or equal to 0.</t>
+          <t>Manufacturer part number or model. Keep this separate from slug and SKU.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>condition</t>
+          <t>sku</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -336,31 +456,31 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Allowed values: new, refurbished. Default: new.</t>
+          <t>Internal stock keeping unit. Must be unique if your database has SKU uniqueness enabled.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>stock_status</t>
+          <t>price_kes</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Optional</t>
+          <t>Required</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Allowed values: in_stock, backorder, out_of_stock. Default: in_stock.</t>
+          <t>Whole number in KSh, greater than or equal to 0.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>stock_quantity</t>
+          <t>cost_price_kes</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -370,14 +490,14 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Whole number, greater than or equal to 0. Default: 0.</t>
+          <t>Whole number internal cost in KSh, or blank.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>images</t>
+          <t>supplier_name</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -387,14 +507,14 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Use 1-3 image URLs separated by semicolons, for example image1.jpg;image2.jpg;image3.jpg. Blank uses /product-placeholder.svg.</t>
+          <t>Supplier name as plain text.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>specs</t>
+          <t>supplier_lead_time_days</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -404,24 +524,160 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Use semicolon-separated Key: Value pairs.</t>
+          <t>Whole number lead time in days, or blank.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
+          <t>reorder_level</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Whole number minimum stock threshold. Default: 0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>reorder_quantity</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Whole number restock quantity. Default: 0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>condition</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Allowed values: new, refurbished. Default: new.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>stock_status</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Allowed values: in_stock, backorder, out_of_stock. Default: in_stock.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>stock_quantity</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Whole number, greater than or equal to 0. Default: 0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>images</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Use 1-3 image URLs separated by semicolons, for example image1.jpg;image2.jpg;image3.jpg. Blank uses /product-placeholder.svg.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>specs</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Use semicolon-separated Key: Value pairs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
           <t>is_featured</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
         <is>
           <t>Allowed values: true/false, yes/no, 1/0. Default: false.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>is_published</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Allowed values: true/false, yes/no, 1/0. Default: true.</t>
         </is>
       </c>
     </row>

</xml_diff>